<commit_message>
ui: auto deploy 2026-03-18T13:34:27
</commit_message>
<xml_diff>
--- a/app/templates/monthly_schedule_template.xlsx
+++ b/app/templates/monthly_schedule_template.xlsx
@@ -3,14 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="현재_통합_문서"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="25600" windowHeight="26640" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="25600" windowHeight="26640" tabRatio="600" firstSheet="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="출동.잔업 초과수당(2)" sheetId="1" state="hidden" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="본사 스케쥴 양식" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="본사 스케쥴 양식" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'본사 스케쥴 양식'!$A$2:$AK$67</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'본사 스케쥴 양식'!$A$2:$AK$67</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -3421,1672 +3420,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="FFFFFF00"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AA45"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="18"/>
-  <cols>
-    <col width="17.5703125" customWidth="1" style="142" min="1" max="1"/>
-    <col width="17.28515625" customWidth="1" style="142" min="2" max="2"/>
-    <col width="13.140625" customWidth="1" style="141" min="3" max="3"/>
-    <col width="17.28515625" customWidth="1" style="142" min="4" max="4"/>
-    <col width="13.140625" customWidth="1" style="141" min="5" max="5"/>
-    <col width="17.28515625" customWidth="1" style="142" min="6" max="6"/>
-    <col width="13.140625" customWidth="1" style="141" min="7" max="7"/>
-    <col width="17.28515625" customWidth="1" style="142" min="8" max="8"/>
-    <col width="13.140625" customWidth="1" style="141" min="9" max="9"/>
-    <col width="17.28515625" customWidth="1" style="142" min="10" max="10"/>
-    <col width="13.140625" customWidth="1" style="141" min="11" max="11"/>
-    <col width="17.28515625" customWidth="1" style="142" min="12" max="12"/>
-    <col width="13.140625" customWidth="1" style="141" min="13" max="13"/>
-    <col width="17.28515625" customWidth="1" style="142" min="14" max="14"/>
-    <col width="13.140625" customWidth="1" style="141" min="15" max="15"/>
-    <col width="17.28515625" customWidth="1" style="142" min="16" max="16"/>
-    <col width="13.140625" customWidth="1" style="141" min="17" max="17"/>
-    <col width="17.28515625" customWidth="1" style="142" min="18" max="18"/>
-    <col width="13.140625" customWidth="1" style="141" min="19" max="19"/>
-    <col width="17.28515625" customWidth="1" style="142" min="20" max="20"/>
-    <col width="13.140625" customWidth="1" style="141" min="21" max="21"/>
-    <col width="5.28515625" customWidth="1" style="142" min="22" max="22"/>
-    <col width="16.28515625" customWidth="1" style="142" min="23" max="23"/>
-    <col width="18.140625" customWidth="1" style="142" min="24" max="27"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="133" customHeight="1" s="142">
-      <c r="B1" s="155" t="inlineStr">
-        <is>
-          <t>근무자 초과 수당 시트</t>
-        </is>
-      </c>
-      <c r="C1" s="145" t="n"/>
-      <c r="D1" s="145" t="n"/>
-      <c r="E1" s="145" t="n"/>
-      <c r="F1" s="145" t="n"/>
-      <c r="G1" s="145" t="n"/>
-      <c r="H1" s="145" t="n"/>
-      <c r="I1" s="145" t="n"/>
-      <c r="J1" s="145" t="n"/>
-      <c r="K1" s="145" t="n"/>
-      <c r="L1" s="145" t="n"/>
-      <c r="M1" s="145" t="n"/>
-      <c r="N1" s="145" t="n"/>
-      <c r="O1" s="145" t="n"/>
-      <c r="P1" s="145" t="n"/>
-      <c r="Q1" s="145" t="n"/>
-      <c r="R1" s="145" t="n"/>
-      <c r="S1" s="145" t="n"/>
-      <c r="T1" s="145" t="n"/>
-      <c r="U1" s="145" t="n"/>
-      <c r="W1" s="3" t="inlineStr">
-        <is>
-          <t>근무자명</t>
-        </is>
-      </c>
-      <c r="X1" s="20" t="inlineStr">
-        <is>
-          <t>주간 총
-초과시간</t>
-        </is>
-      </c>
-      <c r="Y1" s="20" t="inlineStr">
-        <is>
-          <t>평일 총 근무시간(주간)</t>
-        </is>
-      </c>
-      <c r="Z1" s="20" t="inlineStr">
-        <is>
-          <t>주말/공휴일 총 근무시간(주간)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="37" customHeight="1" s="142">
-      <c r="A2" s="148" t="n"/>
-      <c r="B2" s="11" t="n"/>
-      <c r="C2" s="151" t="n"/>
-      <c r="D2" s="11" t="n"/>
-      <c r="E2" s="151" t="n"/>
-      <c r="F2" s="11" t="n"/>
-      <c r="G2" s="151" t="n"/>
-      <c r="H2" s="11" t="n"/>
-      <c r="I2" s="151" t="n"/>
-      <c r="J2" s="11" t="n"/>
-      <c r="K2" s="151" t="n"/>
-      <c r="L2" s="11" t="n"/>
-      <c r="M2" s="151" t="n"/>
-      <c r="N2" s="11" t="n"/>
-      <c r="O2" s="151" t="n"/>
-      <c r="P2" s="11" t="n"/>
-      <c r="Q2" s="151" t="n"/>
-      <c r="R2" s="11" t="n"/>
-      <c r="S2" s="151" t="n"/>
-      <c r="T2" s="11" t="n"/>
-      <c r="U2" s="151" t="n"/>
-      <c r="W2" s="3">
-        <f>#REF!</f>
-        <v/>
-      </c>
-      <c r="X2" s="156" t="n"/>
-      <c r="Y2" s="157" t="n"/>
-      <c r="Z2" s="157">
-        <f>X2-Y2</f>
-        <v/>
-      </c>
-      <c r="AA2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="37" customHeight="1" s="142">
-      <c r="A3" s="143" t="n"/>
-      <c r="B3" s="158">
-        <f>#REF!</f>
-        <v/>
-      </c>
-      <c r="C3" s="152" t="n"/>
-      <c r="D3" s="159">
-        <f>IF(MONTH(B3+DAY(1))=MONTH(B3)+1,"",B3+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="E3" s="152" t="n"/>
-      <c r="F3" s="159">
-        <f>IF(MONTH(D3+DAY(1))=MONTH(D3)+1,"",D3+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="G3" s="152" t="n"/>
-      <c r="H3" s="159">
-        <f>IF(MONTH(F3+DAY(1))=MONTH(F3)+1,"",F3+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="I3" s="152" t="n"/>
-      <c r="J3" s="159">
-        <f>IF(MONTH(H3+DAY(1))=MONTH(H3)+1,"",H3+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="K3" s="152" t="n"/>
-      <c r="L3" s="159">
-        <f>IF(MONTH(J3+DAY(1))=MONTH(J3)+1,"",J3+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="M3" s="152" t="n"/>
-      <c r="N3" s="159">
-        <f>IF(MONTH(L3+DAY(1))=MONTH(L3)+1,"",L3+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="O3" s="152" t="n"/>
-      <c r="P3" s="159">
-        <f>IF(MONTH(N3+DAY(1))=MONTH(N3)+1,"",N3+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="Q3" s="152" t="n"/>
-      <c r="R3" s="159">
-        <f>IF(MONTH(P3+DAY(1))=MONTH(P3)+1,"",P3+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="S3" s="152" t="n"/>
-      <c r="T3" s="159">
-        <f>IF(MONTH(R3+DAY(1))=MONTH(R3)+1,"",R3+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="U3" s="152" t="n"/>
-      <c r="W3" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X3" s="156" t="n"/>
-      <c r="Y3" s="157" t="n"/>
-      <c r="Z3" s="157">
-        <f>X3-Y3</f>
-        <v/>
-      </c>
-      <c r="AA3" s="2" t="n"/>
-    </row>
-    <row r="4" ht="40" customHeight="1" s="142">
-      <c r="A4" s="143" t="n"/>
-      <c r="B4" s="14">
-        <f>TEXT(B3, "ddd")</f>
-        <v/>
-      </c>
-      <c r="C4" s="150" t="n"/>
-      <c r="D4" s="14">
-        <f>TEXT(D3, "ddd")</f>
-        <v/>
-      </c>
-      <c r="E4" s="150" t="n"/>
-      <c r="F4" s="14">
-        <f>TEXT(F3, "ddd")</f>
-        <v/>
-      </c>
-      <c r="G4" s="150" t="n"/>
-      <c r="H4" s="14">
-        <f>TEXT(H3, "ddd")</f>
-        <v/>
-      </c>
-      <c r="I4" s="150" t="n"/>
-      <c r="J4" s="14">
-        <f>TEXT(J3, "ddd")</f>
-        <v/>
-      </c>
-      <c r="K4" s="150" t="n"/>
-      <c r="L4" s="14">
-        <f>TEXT(L3, "ddd")</f>
-        <v/>
-      </c>
-      <c r="M4" s="150" t="n"/>
-      <c r="N4" s="14">
-        <f>TEXT(N3, "ddd")</f>
-        <v/>
-      </c>
-      <c r="O4" s="150" t="n"/>
-      <c r="P4" s="14">
-        <f>TEXT(P3, "ddd")</f>
-        <v/>
-      </c>
-      <c r="Q4" s="150" t="n"/>
-      <c r="R4" s="14">
-        <f>TEXT(R3, "ddd")</f>
-        <v/>
-      </c>
-      <c r="S4" s="150" t="n"/>
-      <c r="T4" s="14">
-        <f>TEXT(T3, "ddd")</f>
-        <v/>
-      </c>
-      <c r="U4" s="150" t="n"/>
-      <c r="W4" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X4" s="156" t="n"/>
-      <c r="Y4" s="157" t="n"/>
-      <c r="Z4" s="157">
-        <f>X4-Y4</f>
-        <v/>
-      </c>
-      <c r="AA4" s="2" t="n"/>
-    </row>
-    <row r="5" ht="42" customHeight="1" s="142">
-      <c r="A5" s="143" t="n"/>
-      <c r="B5" s="21" t="n"/>
-      <c r="C5" s="1" t="n"/>
-      <c r="D5" s="21" t="n"/>
-      <c r="E5" s="1" t="n"/>
-      <c r="F5" s="21" t="n"/>
-      <c r="G5" s="1" t="n"/>
-      <c r="H5" s="21" t="n"/>
-      <c r="I5" s="1" t="n"/>
-      <c r="J5" s="21" t="n"/>
-      <c r="K5" s="1" t="n"/>
-      <c r="L5" s="21" t="n"/>
-      <c r="M5" s="1" t="n"/>
-      <c r="N5" s="21" t="n"/>
-      <c r="O5" s="1" t="n"/>
-      <c r="P5" s="21" t="n"/>
-      <c r="Q5" s="1" t="n"/>
-      <c r="R5" s="21" t="n"/>
-      <c r="S5" s="1" t="n"/>
-      <c r="T5" s="21" t="n"/>
-      <c r="U5" s="1" t="n"/>
-      <c r="W5" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X5" s="156" t="n"/>
-      <c r="Y5" s="157" t="n"/>
-      <c r="Z5" s="157">
-        <f>X5-Y5</f>
-        <v/>
-      </c>
-      <c r="AA5" s="2" t="n"/>
-    </row>
-    <row r="6" ht="42" customHeight="1" s="142">
-      <c r="A6" s="143" t="n"/>
-      <c r="B6" s="21" t="n"/>
-      <c r="C6" s="1" t="n"/>
-      <c r="D6" s="21" t="n"/>
-      <c r="E6" s="1" t="n"/>
-      <c r="F6" s="21" t="n"/>
-      <c r="G6" s="1" t="n"/>
-      <c r="H6" s="21" t="n"/>
-      <c r="I6" s="1" t="n"/>
-      <c r="J6" s="21" t="n"/>
-      <c r="K6" s="1" t="n"/>
-      <c r="L6" s="21" t="n"/>
-      <c r="M6" s="1" t="n"/>
-      <c r="N6" s="21" t="n"/>
-      <c r="O6" s="1" t="n"/>
-      <c r="P6" s="6" t="n"/>
-      <c r="Q6" s="1" t="n"/>
-      <c r="R6" s="6" t="n"/>
-      <c r="S6" s="1" t="n"/>
-      <c r="T6" s="6" t="n"/>
-      <c r="U6" s="1" t="n"/>
-      <c r="W6" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X6" s="156" t="n"/>
-      <c r="Y6" s="157" t="n"/>
-      <c r="Z6" s="157">
-        <f>X6-Y6</f>
-        <v/>
-      </c>
-      <c r="AA6" s="2" t="n"/>
-    </row>
-    <row r="7" ht="42" customHeight="1" s="142">
-      <c r="A7" s="143" t="n"/>
-      <c r="B7" s="21" t="n"/>
-      <c r="C7" s="1" t="n"/>
-      <c r="D7" s="21" t="n"/>
-      <c r="E7" s="1" t="n"/>
-      <c r="F7" s="21" t="n"/>
-      <c r="G7" s="1" t="n"/>
-      <c r="H7" s="21" t="n"/>
-      <c r="I7" s="1" t="n"/>
-      <c r="J7" s="21" t="n"/>
-      <c r="K7" s="1" t="n"/>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="1" t="n"/>
-      <c r="N7" s="7" t="n"/>
-      <c r="O7" s="1" t="n"/>
-      <c r="P7" s="6" t="n"/>
-      <c r="Q7" s="1" t="n"/>
-      <c r="R7" s="6" t="n"/>
-      <c r="S7" s="1" t="n"/>
-      <c r="T7" s="6" t="n"/>
-      <c r="U7" s="1" t="n"/>
-      <c r="W7" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X7" s="156" t="n"/>
-      <c r="Y7" s="157" t="n"/>
-      <c r="Z7" s="157">
-        <f>X7-Y7</f>
-        <v/>
-      </c>
-      <c r="AA7" s="2" t="n"/>
-    </row>
-    <row r="8" ht="42" customHeight="1" s="142">
-      <c r="A8" s="143" t="n"/>
-      <c r="B8" s="21" t="n"/>
-      <c r="C8" s="1" t="n"/>
-      <c r="D8" s="21" t="n"/>
-      <c r="E8" s="1" t="n"/>
-      <c r="F8" s="21" t="n"/>
-      <c r="G8" s="1" t="n"/>
-      <c r="H8" s="21" t="n"/>
-      <c r="I8" s="1" t="n"/>
-      <c r="J8" s="21" t="n"/>
-      <c r="K8" s="1" t="n"/>
-      <c r="L8" s="21" t="n"/>
-      <c r="M8" s="1" t="n"/>
-      <c r="N8" s="21" t="n"/>
-      <c r="O8" s="1" t="n"/>
-      <c r="P8" s="6" t="n"/>
-      <c r="Q8" s="1" t="n"/>
-      <c r="R8" s="6" t="n"/>
-      <c r="S8" s="1" t="n"/>
-      <c r="T8" s="6" t="n"/>
-      <c r="U8" s="1" t="n"/>
-      <c r="W8" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X8" s="156" t="n"/>
-      <c r="Y8" s="157" t="n"/>
-      <c r="Z8" s="157">
-        <f>X8-Y8</f>
-        <v/>
-      </c>
-      <c r="AA8" s="2" t="n"/>
-    </row>
-    <row r="9" ht="42" customHeight="1" s="142">
-      <c r="A9" s="146" t="n"/>
-      <c r="B9" s="21" t="n"/>
-      <c r="C9" s="1" t="n"/>
-      <c r="D9" s="21" t="n"/>
-      <c r="E9" s="1" t="n"/>
-      <c r="F9" s="21" t="n"/>
-      <c r="G9" s="1" t="n"/>
-      <c r="H9" s="21" t="n"/>
-      <c r="I9" s="1" t="n"/>
-      <c r="J9" s="21" t="n"/>
-      <c r="K9" s="1" t="n"/>
-      <c r="L9" s="21" t="n"/>
-      <c r="M9" s="1" t="n"/>
-      <c r="N9" s="21" t="n"/>
-      <c r="O9" s="1" t="n"/>
-      <c r="P9" s="6" t="n"/>
-      <c r="Q9" s="1" t="n"/>
-      <c r="R9" s="6" t="n"/>
-      <c r="S9" s="1" t="n"/>
-      <c r="T9" s="6" t="n"/>
-      <c r="U9" s="1" t="n"/>
-      <c r="W9" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X9" s="156" t="n"/>
-      <c r="Y9" s="157" t="n"/>
-      <c r="Z9" s="157">
-        <f>X9-Y9</f>
-        <v/>
-      </c>
-      <c r="AA9" s="2" t="n"/>
-    </row>
-    <row r="10" ht="216" customHeight="1" s="142">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>근무 사유</t>
-        </is>
-      </c>
-      <c r="B10" s="159" t="n"/>
-      <c r="C10" s="81" t="n"/>
-      <c r="D10" s="159" t="n"/>
-      <c r="E10" s="81" t="n"/>
-      <c r="F10" s="159" t="n"/>
-      <c r="G10" s="81" t="n"/>
-      <c r="H10" s="159" t="n"/>
-      <c r="I10" s="81" t="n"/>
-      <c r="J10" s="159" t="n"/>
-      <c r="K10" s="81" t="n"/>
-      <c r="L10" s="159" t="n"/>
-      <c r="M10" s="81" t="n"/>
-      <c r="N10" s="159" t="n"/>
-      <c r="O10" s="81" t="n"/>
-      <c r="P10" s="159" t="n"/>
-      <c r="Q10" s="81" t="n"/>
-      <c r="R10" s="159" t="n"/>
-      <c r="S10" s="81" t="n"/>
-      <c r="T10" s="159" t="n"/>
-      <c r="U10" s="81" t="n"/>
-      <c r="W10" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X10" s="156" t="n"/>
-      <c r="Y10" s="157" t="n"/>
-      <c r="Z10" s="157">
-        <f>X10-Y10</f>
-        <v/>
-      </c>
-      <c r="AA10" s="2" t="n"/>
-    </row>
-    <row r="11" ht="37" customHeight="1" s="142">
-      <c r="A11" s="153" t="n"/>
-      <c r="B11" s="159">
-        <f>IF(MONTH(T3+DAY(1))=MONTH(T3)+1,"",T3+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="C11" s="160" t="n"/>
-      <c r="D11" s="159">
-        <f>IF(MONTH(B11+DAY(1))=MONTH(B11)+1,"",B11+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="E11" s="160" t="n"/>
-      <c r="F11" s="159">
-        <f>IF(MONTH(D11+DAY(1))=MONTH(D11)+1,"",D11+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="G11" s="160" t="n"/>
-      <c r="H11" s="159">
-        <f>IF(MONTH(F11+DAY(1))=MONTH(F11)+1,"",F11+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="I11" s="160" t="n"/>
-      <c r="J11" s="159">
-        <f>IF(MONTH(H11+DAY(1))=MONTH(H11)+1,"",H11+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="K11" s="160" t="n"/>
-      <c r="L11" s="159">
-        <f>IF(MONTH(J11+DAY(1))=MONTH(J11)+1,"",J11+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="M11" s="160" t="n"/>
-      <c r="N11" s="159">
-        <f>IF(MONTH(L11+DAY(1))=MONTH(L11)+1,"",L11+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="O11" s="160" t="n"/>
-      <c r="P11" s="159">
-        <f>IF(MONTH(N11+DAY(1))=MONTH(N11)+1,"",N11+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="Q11" s="160" t="n"/>
-      <c r="R11" s="159">
-        <f>IF(MONTH(P11+DAY(1))=MONTH(P11)+1,"",P11+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="S11" s="160" t="n"/>
-      <c r="T11" s="159">
-        <f>IF(MONTH(R11+DAY(1))=MONTH(R11)+1,"",R11+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="U11" s="160" t="n"/>
-      <c r="W11" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X11" s="156" t="n"/>
-      <c r="Y11" s="157" t="n"/>
-      <c r="Z11" s="157">
-        <f>X11-Y11</f>
-        <v/>
-      </c>
-      <c r="AA11" s="2" t="n"/>
-    </row>
-    <row r="12" ht="28" customHeight="1" s="142">
-      <c r="A12" s="143" t="n"/>
-      <c r="B12" s="14">
-        <f>TEXT(B11, "ddd")</f>
-        <v/>
-      </c>
-      <c r="C12" s="150" t="n"/>
-      <c r="D12" s="14">
-        <f>TEXT(D11, "ddd")</f>
-        <v/>
-      </c>
-      <c r="E12" s="150" t="n"/>
-      <c r="F12" s="14">
-        <f>TEXT(F11, "ddd")</f>
-        <v/>
-      </c>
-      <c r="G12" s="150" t="n"/>
-      <c r="H12" s="14">
-        <f>TEXT(H11, "ddd")</f>
-        <v/>
-      </c>
-      <c r="I12" s="150" t="n"/>
-      <c r="J12" s="14">
-        <f>TEXT(J11, "ddd")</f>
-        <v/>
-      </c>
-      <c r="K12" s="150" t="n"/>
-      <c r="L12" s="14">
-        <f>TEXT(L11, "ddd")</f>
-        <v/>
-      </c>
-      <c r="M12" s="150" t="n"/>
-      <c r="N12" s="14">
-        <f>TEXT(N11, "ddd")</f>
-        <v/>
-      </c>
-      <c r="O12" s="150" t="n"/>
-      <c r="P12" s="14">
-        <f>TEXT(P11, "ddd")</f>
-        <v/>
-      </c>
-      <c r="Q12" s="150" t="n"/>
-      <c r="R12" s="14">
-        <f>TEXT(R11, "ddd")</f>
-        <v/>
-      </c>
-      <c r="S12" s="150" t="n"/>
-      <c r="T12" s="14">
-        <f>TEXT(T11, "ddd")</f>
-        <v/>
-      </c>
-      <c r="U12" s="150" t="n"/>
-      <c r="W12" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X12" s="156" t="n"/>
-      <c r="Y12" s="157" t="n"/>
-      <c r="Z12" s="157">
-        <f>X12-Y12</f>
-        <v/>
-      </c>
-      <c r="AA12" s="2" t="n"/>
-    </row>
-    <row r="13" ht="42" customHeight="1" s="142">
-      <c r="A13" s="143" t="n"/>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="21" t="n"/>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="21" t="n"/>
-      <c r="G13" s="8" t="n"/>
-      <c r="H13" s="21" t="n"/>
-      <c r="I13" s="8" t="n"/>
-      <c r="J13" s="21" t="n"/>
-      <c r="K13" s="8" t="n"/>
-      <c r="L13" s="21" t="n"/>
-      <c r="M13" s="8" t="n"/>
-      <c r="N13" s="21" t="n"/>
-      <c r="O13" s="8" t="n"/>
-      <c r="P13" s="6" t="n"/>
-      <c r="Q13" s="8" t="n"/>
-      <c r="R13" s="6" t="n"/>
-      <c r="S13" s="8" t="n"/>
-      <c r="T13" s="6" t="n"/>
-      <c r="U13" s="8" t="n"/>
-      <c r="W13" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X13" s="156" t="n"/>
-      <c r="Y13" s="157" t="n"/>
-      <c r="Z13" s="157">
-        <f>X13-Y13</f>
-        <v/>
-      </c>
-      <c r="AA13" s="2" t="n"/>
-    </row>
-    <row r="14" ht="42" customHeight="1" s="142">
-      <c r="A14" s="143" t="n"/>
-      <c r="B14" s="21" t="n"/>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="21" t="n"/>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="21" t="n"/>
-      <c r="G14" s="8" t="n"/>
-      <c r="H14" s="21" t="n"/>
-      <c r="I14" s="8" t="n"/>
-      <c r="J14" s="21" t="n"/>
-      <c r="K14" s="8" t="n"/>
-      <c r="L14" s="21" t="n"/>
-      <c r="M14" s="8" t="n"/>
-      <c r="N14" s="21" t="n"/>
-      <c r="O14" s="8" t="n"/>
-      <c r="P14" s="6" t="n"/>
-      <c r="Q14" s="8" t="n"/>
-      <c r="R14" s="6" t="n"/>
-      <c r="S14" s="8" t="n"/>
-      <c r="T14" s="6" t="n"/>
-      <c r="U14" s="8" t="n"/>
-      <c r="W14" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X14" s="156" t="n"/>
-      <c r="Y14" s="157" t="n"/>
-      <c r="Z14" s="157">
-        <f>X14-Y14</f>
-        <v/>
-      </c>
-      <c r="AA14" s="2" t="n"/>
-    </row>
-    <row r="15" ht="42" customHeight="1" s="142">
-      <c r="A15" s="143" t="n"/>
-      <c r="B15" s="21" t="n"/>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="21" t="n"/>
-      <c r="E15" s="8" t="n"/>
-      <c r="F15" s="21" t="n"/>
-      <c r="G15" s="8" t="n"/>
-      <c r="H15" s="21" t="n"/>
-      <c r="I15" s="8" t="n"/>
-      <c r="J15" s="21" t="n"/>
-      <c r="K15" s="8" t="n"/>
-      <c r="L15" s="21" t="n"/>
-      <c r="M15" s="8" t="n"/>
-      <c r="N15" s="21" t="n"/>
-      <c r="O15" s="8" t="n"/>
-      <c r="P15" s="6" t="n"/>
-      <c r="Q15" s="8" t="n"/>
-      <c r="R15" s="6" t="n"/>
-      <c r="S15" s="8" t="n"/>
-      <c r="T15" s="6" t="n"/>
-      <c r="U15" s="8" t="n"/>
-      <c r="W15" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X15" s="156" t="n"/>
-      <c r="Y15" s="157" t="n"/>
-      <c r="Z15" s="157">
-        <f>X15-Y15</f>
-        <v/>
-      </c>
-      <c r="AA15" s="2" t="n"/>
-    </row>
-    <row r="16" ht="42" customHeight="1" s="142">
-      <c r="A16" s="143" t="n"/>
-      <c r="B16" s="21" t="n"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="21" t="n"/>
-      <c r="E16" s="8" t="n"/>
-      <c r="F16" s="21" t="n"/>
-      <c r="G16" s="8" t="n"/>
-      <c r="H16" s="21" t="n"/>
-      <c r="I16" s="8" t="n"/>
-      <c r="J16" s="21" t="n"/>
-      <c r="K16" s="8" t="n"/>
-      <c r="L16" s="21" t="n"/>
-      <c r="M16" s="8" t="n"/>
-      <c r="N16" s="21" t="n"/>
-      <c r="O16" s="8" t="n"/>
-      <c r="P16" s="6" t="n"/>
-      <c r="Q16" s="8" t="n"/>
-      <c r="R16" s="6" t="n"/>
-      <c r="S16" s="8" t="n"/>
-      <c r="T16" s="6" t="n"/>
-      <c r="U16" s="8" t="n"/>
-      <c r="W16" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X16" s="156" t="n"/>
-      <c r="Y16" s="157" t="n"/>
-      <c r="Z16" s="157">
-        <f>X16-Y16</f>
-        <v/>
-      </c>
-      <c r="AA16" s="2" t="n"/>
-    </row>
-    <row r="17" ht="42" customHeight="1" s="142">
-      <c r="A17" s="146" t="n"/>
-      <c r="B17" s="161" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="161" t="n"/>
-      <c r="E17" s="8" t="n"/>
-      <c r="F17" s="161" t="n"/>
-      <c r="G17" s="8" t="n"/>
-      <c r="H17" s="161" t="n"/>
-      <c r="I17" s="8" t="n"/>
-      <c r="J17" s="161" t="n"/>
-      <c r="K17" s="8" t="n"/>
-      <c r="L17" s="161" t="n"/>
-      <c r="M17" s="8" t="n"/>
-      <c r="N17" s="161" t="n"/>
-      <c r="O17" s="8" t="n"/>
-      <c r="P17" s="6" t="n"/>
-      <c r="Q17" s="8" t="n"/>
-      <c r="R17" s="6" t="n"/>
-      <c r="S17" s="8" t="n"/>
-      <c r="T17" s="6" t="n"/>
-      <c r="U17" s="8" t="n"/>
-      <c r="W17" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X17" s="156" t="n"/>
-      <c r="Y17" s="157" t="n"/>
-      <c r="Z17" s="157">
-        <f>X17-Y17</f>
-        <v/>
-      </c>
-      <c r="AA17" s="2" t="n"/>
-    </row>
-    <row r="18" ht="216" customHeight="1" s="142">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>근무 사유</t>
-        </is>
-      </c>
-      <c r="B18" s="159" t="n"/>
-      <c r="C18" s="81" t="n"/>
-      <c r="D18" s="159" t="n"/>
-      <c r="E18" s="81" t="n"/>
-      <c r="F18" s="159" t="n"/>
-      <c r="G18" s="81" t="n"/>
-      <c r="H18" s="159" t="n"/>
-      <c r="I18" s="81" t="n"/>
-      <c r="J18" s="159" t="n"/>
-      <c r="K18" s="81" t="n"/>
-      <c r="L18" s="159" t="n"/>
-      <c r="M18" s="81" t="n"/>
-      <c r="N18" s="159" t="n"/>
-      <c r="O18" s="81" t="n"/>
-      <c r="P18" s="159" t="n"/>
-      <c r="Q18" s="81" t="n"/>
-      <c r="R18" s="159" t="n"/>
-      <c r="S18" s="81" t="n"/>
-      <c r="T18" s="159" t="n"/>
-      <c r="U18" s="81" t="n"/>
-      <c r="W18" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X18" s="156" t="n"/>
-      <c r="Y18" s="157" t="n"/>
-      <c r="Z18" s="157">
-        <f>X18-Y18</f>
-        <v/>
-      </c>
-      <c r="AA18" s="2" t="n"/>
-    </row>
-    <row r="19" ht="37" customHeight="1" s="142">
-      <c r="A19" s="153" t="n"/>
-      <c r="B19" s="159">
-        <f>IF(MONTH(T11+DAY(1))=MONTH(T11)+1,"",T11+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="C19" s="160" t="n"/>
-      <c r="D19" s="159">
-        <f>IF(MONTH(B19+DAY(1))=MONTH(B19)+1,"",B19+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="E19" s="160" t="n"/>
-      <c r="F19" s="159">
-        <f>IF(MONTH(D19+DAY(1))=MONTH(D19)+1,"",D19+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="G19" s="160" t="n"/>
-      <c r="H19" s="159">
-        <f>IF(MONTH(F19+DAY(1))=MONTH(F19)+1,"",F19+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="I19" s="160" t="n"/>
-      <c r="J19" s="159">
-        <f>IF(MONTH(H19+DAY(1))=MONTH(H19)+1,"",H19+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="K19" s="160" t="n"/>
-      <c r="L19" s="159">
-        <f>IF(MONTH(J19+DAY(1))=MONTH(J19)+1,"",J19+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="M19" s="160" t="n"/>
-      <c r="N19" s="159">
-        <f>IF(MONTH(L19+DAY(1))=MONTH(L19)+1,"",L19+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="O19" s="160" t="n"/>
-      <c r="P19" s="159">
-        <f>IF(MONTH(N19+DAY(1))=MONTH(N19)+1,"",N19+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="Q19" s="160" t="n"/>
-      <c r="R19" s="159">
-        <f>IF(MONTH(P19+DAY(1))=MONTH(P19)+1,"",P19+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="S19" s="160" t="n"/>
-      <c r="T19" s="159">
-        <f>IF(MONTH(R19+DAY(1))=MONTH(R19)+1,"",R19+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="U19" s="160" t="n"/>
-      <c r="W19" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X19" s="156" t="n"/>
-      <c r="Y19" s="157" t="n"/>
-      <c r="Z19" s="157">
-        <f>X19-Y19</f>
-        <v/>
-      </c>
-      <c r="AA19" s="2" t="n"/>
-    </row>
-    <row r="20" ht="28" customHeight="1" s="142">
-      <c r="A20" s="143" t="n"/>
-      <c r="B20" s="14">
-        <f>TEXT(B19, "ddd")</f>
-        <v/>
-      </c>
-      <c r="C20" s="150" t="n"/>
-      <c r="D20" s="14">
-        <f>TEXT(D19, "ddd")</f>
-        <v/>
-      </c>
-      <c r="E20" s="150" t="n"/>
-      <c r="F20" s="14">
-        <f>TEXT(F19, "ddd")</f>
-        <v/>
-      </c>
-      <c r="G20" s="150" t="n"/>
-      <c r="H20" s="14">
-        <f>TEXT(H19, "ddd")</f>
-        <v/>
-      </c>
-      <c r="I20" s="150" t="n"/>
-      <c r="J20" s="14">
-        <f>TEXT(J19, "ddd")</f>
-        <v/>
-      </c>
-      <c r="K20" s="150" t="n"/>
-      <c r="L20" s="14">
-        <f>TEXT(L19, "ddd")</f>
-        <v/>
-      </c>
-      <c r="M20" s="150" t="n"/>
-      <c r="N20" s="14">
-        <f>TEXT(N19, "ddd")</f>
-        <v/>
-      </c>
-      <c r="O20" s="150" t="n"/>
-      <c r="P20" s="14">
-        <f>TEXT(P19, "ddd")</f>
-        <v/>
-      </c>
-      <c r="Q20" s="150" t="n"/>
-      <c r="R20" s="14">
-        <f>TEXT(R19, "ddd")</f>
-        <v/>
-      </c>
-      <c r="S20" s="150" t="n"/>
-      <c r="T20" s="14">
-        <f>TEXT(T19, "ddd")</f>
-        <v/>
-      </c>
-      <c r="U20" s="150" t="n"/>
-      <c r="W20" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X20" s="156" t="n"/>
-      <c r="Y20" s="157" t="n"/>
-      <c r="Z20" s="157">
-        <f>X20-Y20</f>
-        <v/>
-      </c>
-      <c r="AA20" s="2" t="n"/>
-    </row>
-    <row r="21" ht="42" customHeight="1" s="142">
-      <c r="A21" s="143" t="n"/>
-      <c r="B21" s="21" t="n"/>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="21" t="n"/>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="21" t="n"/>
-      <c r="G21" s="8" t="n"/>
-      <c r="H21" s="21" t="n"/>
-      <c r="I21" s="8" t="n"/>
-      <c r="J21" s="21" t="n"/>
-      <c r="K21" s="8" t="n"/>
-      <c r="L21" s="21" t="n"/>
-      <c r="M21" s="8" t="n"/>
-      <c r="N21" s="21" t="n"/>
-      <c r="O21" s="8" t="n"/>
-      <c r="P21" s="6" t="n"/>
-      <c r="Q21" s="8" t="n"/>
-      <c r="R21" s="6" t="n"/>
-      <c r="S21" s="8" t="n"/>
-      <c r="T21" s="6" t="n"/>
-      <c r="U21" s="8" t="n"/>
-      <c r="W21" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X21" s="156" t="n"/>
-      <c r="Y21" s="157" t="n"/>
-      <c r="Z21" s="157">
-        <f>X21-Y21</f>
-        <v/>
-      </c>
-      <c r="AA21" s="2" t="n"/>
-    </row>
-    <row r="22" ht="42" customHeight="1" s="142">
-      <c r="A22" s="143" t="n"/>
-      <c r="B22" s="21" t="n"/>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="21" t="n"/>
-      <c r="E22" s="8" t="n"/>
-      <c r="F22" s="21" t="n"/>
-      <c r="G22" s="8" t="n"/>
-      <c r="H22" s="21" t="n"/>
-      <c r="I22" s="8" t="n"/>
-      <c r="J22" s="21" t="n"/>
-      <c r="K22" s="8" t="n"/>
-      <c r="L22" s="21" t="n"/>
-      <c r="M22" s="8" t="n"/>
-      <c r="N22" s="21" t="n"/>
-      <c r="O22" s="8" t="n"/>
-      <c r="P22" s="6" t="n"/>
-      <c r="Q22" s="8" t="n"/>
-      <c r="R22" s="6" t="n"/>
-      <c r="S22" s="8" t="n"/>
-      <c r="T22" s="6" t="n"/>
-      <c r="U22" s="8" t="n"/>
-      <c r="W22" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X22" s="156" t="n"/>
-      <c r="Y22" s="157" t="n"/>
-      <c r="Z22" s="157">
-        <f>X22-Y22</f>
-        <v/>
-      </c>
-      <c r="AA22" s="2" t="n"/>
-    </row>
-    <row r="23" ht="42" customHeight="1" s="142">
-      <c r="A23" s="143" t="n"/>
-      <c r="B23" s="21" t="n"/>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="21" t="n"/>
-      <c r="E23" s="8" t="n"/>
-      <c r="F23" s="21" t="n"/>
-      <c r="G23" s="8" t="n"/>
-      <c r="H23" s="21" t="n"/>
-      <c r="I23" s="8" t="n"/>
-      <c r="J23" s="21" t="n"/>
-      <c r="K23" s="8" t="n"/>
-      <c r="L23" s="21" t="n"/>
-      <c r="M23" s="8" t="n"/>
-      <c r="N23" s="21" t="n"/>
-      <c r="O23" s="8" t="n"/>
-      <c r="P23" s="6" t="n"/>
-      <c r="Q23" s="8" t="n"/>
-      <c r="R23" s="6" t="n"/>
-      <c r="S23" s="8" t="n"/>
-      <c r="T23" s="6" t="n"/>
-      <c r="U23" s="8" t="n"/>
-      <c r="W23" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X23" s="156" t="n"/>
-      <c r="Y23" s="157" t="n"/>
-      <c r="Z23" s="157">
-        <f>X23-Y23</f>
-        <v/>
-      </c>
-      <c r="AA23" s="2" t="n"/>
-    </row>
-    <row r="24" ht="42" customHeight="1" s="142">
-      <c r="A24" s="143" t="n"/>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="8" t="n"/>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="8" t="n"/>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="8" t="n"/>
-      <c r="J24" s="3" t="n"/>
-      <c r="K24" s="8" t="n"/>
-      <c r="L24" s="3" t="n"/>
-      <c r="M24" s="8" t="n"/>
-      <c r="N24" s="3" t="n"/>
-      <c r="O24" s="8" t="n"/>
-      <c r="P24" s="7" t="n"/>
-      <c r="Q24" s="8" t="n"/>
-      <c r="R24" s="7" t="n"/>
-      <c r="S24" s="8" t="n"/>
-      <c r="T24" s="7" t="n"/>
-      <c r="U24" s="8" t="n"/>
-      <c r="W24" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X24" s="156" t="n"/>
-      <c r="Y24" s="157" t="n"/>
-      <c r="Z24" s="157">
-        <f>X24-Y24</f>
-        <v/>
-      </c>
-      <c r="AA24" s="2" t="n"/>
-    </row>
-    <row r="25" ht="42" customHeight="1" s="142">
-      <c r="A25" s="146" t="n"/>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="8" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="8" t="n"/>
-      <c r="H25" s="3" t="n"/>
-      <c r="I25" s="8" t="n"/>
-      <c r="J25" s="3" t="n"/>
-      <c r="K25" s="8" t="n"/>
-      <c r="L25" s="3" t="n"/>
-      <c r="M25" s="8" t="n"/>
-      <c r="N25" s="3" t="n"/>
-      <c r="O25" s="8" t="n"/>
-      <c r="P25" s="7" t="n"/>
-      <c r="Q25" s="8" t="n"/>
-      <c r="R25" s="7" t="n"/>
-      <c r="S25" s="8" t="n"/>
-      <c r="T25" s="7" t="n"/>
-      <c r="U25" s="8" t="n"/>
-      <c r="W25" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X25" s="156" t="n"/>
-      <c r="Y25" s="157" t="n"/>
-      <c r="Z25" s="157">
-        <f>X25-Y25</f>
-        <v/>
-      </c>
-      <c r="AA25" s="2" t="n"/>
-    </row>
-    <row r="26" ht="216" customHeight="1" s="142">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>근무 사유</t>
-        </is>
-      </c>
-      <c r="B26" s="159" t="n"/>
-      <c r="C26" s="81" t="n"/>
-      <c r="D26" s="159" t="n"/>
-      <c r="E26" s="81" t="n"/>
-      <c r="F26" s="159" t="n"/>
-      <c r="G26" s="81" t="n"/>
-      <c r="H26" s="159" t="n"/>
-      <c r="I26" s="81" t="n"/>
-      <c r="J26" s="159" t="n"/>
-      <c r="K26" s="81" t="n"/>
-      <c r="L26" s="159" t="n"/>
-      <c r="M26" s="81" t="n"/>
-      <c r="N26" s="159" t="n"/>
-      <c r="O26" s="81" t="n"/>
-      <c r="P26" s="159" t="n"/>
-      <c r="Q26" s="81" t="n"/>
-      <c r="R26" s="159" t="n"/>
-      <c r="S26" s="81" t="n"/>
-      <c r="T26" s="159" t="n"/>
-      <c r="U26" s="81" t="n"/>
-      <c r="W26" s="3">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-      <c r="X26" s="156" t="n"/>
-      <c r="Y26" s="157" t="n"/>
-      <c r="Z26" s="157">
-        <f>X26-Y26</f>
-        <v/>
-      </c>
-      <c r="AA26" s="2" t="n"/>
-    </row>
-    <row r="27" ht="37" customHeight="1" s="142">
-      <c r="A27" s="153" t="n"/>
-      <c r="B27" s="159">
-        <f>IF(MONTH(T19+DAY(1))=MONTH(T19)+1,"",T19+DAY(1))</f>
-        <v/>
-      </c>
-      <c r="C27" s="160" t="n"/>
-      <c r="D27" s="159" t="n"/>
-      <c r="E27" s="162" t="n"/>
-      <c r="F27" s="15" t="n"/>
-      <c r="G27" s="17" t="n"/>
-      <c r="H27" s="15" t="n"/>
-      <c r="I27" s="17" t="n"/>
-      <c r="J27" s="15" t="n"/>
-      <c r="K27" s="17" t="n"/>
-      <c r="L27" s="15" t="n"/>
-      <c r="M27" s="17" t="n"/>
-      <c r="N27" s="15" t="n"/>
-      <c r="O27" s="17" t="n"/>
-      <c r="P27" s="15" t="n"/>
-      <c r="Q27" s="17" t="n"/>
-      <c r="R27" s="15" t="n"/>
-      <c r="S27" s="17" t="n"/>
-      <c r="T27" s="15" t="n"/>
-      <c r="U27" s="17" t="n"/>
-      <c r="W27" s="0">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="28" customHeight="1" s="142">
-      <c r="A28" s="143" t="n"/>
-      <c r="B28" s="18">
-        <f>TEXT(B27, "ddd")</f>
-        <v/>
-      </c>
-      <c r="C28" s="150" t="n"/>
-      <c r="D28" s="18" t="n"/>
-      <c r="E28" s="19" t="n"/>
-      <c r="F28" s="15" t="n"/>
-      <c r="G28" s="17" t="n"/>
-      <c r="H28" s="15" t="n"/>
-      <c r="I28" s="17" t="n"/>
-      <c r="J28" s="15" t="n"/>
-      <c r="K28" s="17" t="n"/>
-      <c r="L28" s="15" t="n"/>
-      <c r="M28" s="17" t="n"/>
-      <c r="N28" s="15" t="n"/>
-      <c r="O28" s="17" t="n"/>
-      <c r="P28" s="15" t="n"/>
-      <c r="Q28" s="17" t="n"/>
-      <c r="R28" s="15" t="n"/>
-      <c r="S28" s="17" t="n"/>
-      <c r="T28" s="15" t="n"/>
-      <c r="U28" s="17" t="n"/>
-      <c r="W28" s="0">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="42" customHeight="1" s="142">
-      <c r="A29" s="143" t="n"/>
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="7" t="n"/>
-      <c r="E29" s="9" t="n"/>
-      <c r="F29" s="7" t="n"/>
-      <c r="G29" s="9" t="n"/>
-      <c r="H29" s="7" t="n"/>
-      <c r="I29" s="9" t="n"/>
-      <c r="J29" s="7" t="n"/>
-      <c r="K29" s="9" t="n"/>
-      <c r="L29" s="7" t="n"/>
-      <c r="M29" s="9" t="n"/>
-      <c r="N29" s="7" t="n"/>
-      <c r="O29" s="9" t="n"/>
-      <c r="P29" s="7" t="n"/>
-      <c r="Q29" s="9" t="n"/>
-      <c r="R29" s="7" t="n"/>
-      <c r="S29" s="9" t="n"/>
-      <c r="T29" s="7" t="n"/>
-      <c r="U29" s="9" t="n"/>
-      <c r="W29" s="0">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="42" customHeight="1" s="142">
-      <c r="A30" s="143" t="n"/>
-      <c r="B30" s="7" t="n"/>
-      <c r="C30" s="8" t="n"/>
-      <c r="D30" s="7" t="n"/>
-      <c r="E30" s="9" t="n"/>
-      <c r="F30" s="7" t="n"/>
-      <c r="G30" s="9" t="n"/>
-      <c r="H30" s="7" t="n"/>
-      <c r="I30" s="9" t="n"/>
-      <c r="J30" s="7" t="n"/>
-      <c r="K30" s="9" t="n"/>
-      <c r="L30" s="7" t="n"/>
-      <c r="M30" s="9" t="n"/>
-      <c r="N30" s="7" t="n"/>
-      <c r="O30" s="9" t="n"/>
-      <c r="P30" s="7" t="n"/>
-      <c r="Q30" s="9" t="n"/>
-      <c r="R30" s="7" t="n"/>
-      <c r="S30" s="9" t="n"/>
-      <c r="T30" s="7" t="n"/>
-      <c r="U30" s="9" t="n"/>
-      <c r="W30" s="0">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="42" customHeight="1" s="142">
-      <c r="A31" s="143" t="n"/>
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="8" t="n"/>
-      <c r="D31" s="7" t="n"/>
-      <c r="E31" s="9" t="n"/>
-      <c r="F31" s="7" t="n"/>
-      <c r="G31" s="9" t="n"/>
-      <c r="H31" s="7" t="n"/>
-      <c r="I31" s="9" t="n"/>
-      <c r="J31" s="7" t="n"/>
-      <c r="K31" s="9" t="n"/>
-      <c r="L31" s="7" t="n"/>
-      <c r="M31" s="9" t="n"/>
-      <c r="N31" s="7" t="n"/>
-      <c r="O31" s="9" t="n"/>
-      <c r="P31" s="7" t="n"/>
-      <c r="Q31" s="9" t="n"/>
-      <c r="R31" s="7" t="n"/>
-      <c r="S31" s="9" t="n"/>
-      <c r="T31" s="7" t="n"/>
-      <c r="U31" s="9" t="n"/>
-      <c r="W31" s="0">
-        <f>IF(#REF!="","",#REF!)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="42" customHeight="1" s="142">
-      <c r="A32" s="143" t="n"/>
-      <c r="B32" s="7" t="n"/>
-      <c r="C32" s="8" t="n"/>
-      <c r="D32" s="7" t="n"/>
-      <c r="E32" s="9" t="n"/>
-      <c r="F32" s="7" t="n"/>
-      <c r="G32" s="9" t="n"/>
-      <c r="H32" s="7" t="n"/>
-      <c r="I32" s="9" t="n"/>
-      <c r="J32" s="7" t="n"/>
-      <c r="K32" s="9" t="n"/>
-      <c r="L32" s="7" t="n"/>
-      <c r="M32" s="9" t="n"/>
-      <c r="N32" s="7" t="n"/>
-      <c r="O32" s="9" t="n"/>
-      <c r="P32" s="7" t="n"/>
-      <c r="Q32" s="9" t="n"/>
-      <c r="R32" s="7" t="n"/>
-      <c r="S32" s="9" t="n"/>
-      <c r="T32" s="7" t="n"/>
-      <c r="U32" s="9" t="n"/>
-    </row>
-    <row r="33" ht="42" customHeight="1" s="142">
-      <c r="A33" s="146" t="n"/>
-      <c r="B33" s="7" t="n"/>
-      <c r="C33" s="8" t="n"/>
-      <c r="D33" s="7" t="n"/>
-      <c r="E33" s="9" t="n"/>
-      <c r="F33" s="7" t="n"/>
-      <c r="G33" s="9" t="n"/>
-      <c r="H33" s="7" t="n"/>
-      <c r="I33" s="9" t="n"/>
-      <c r="J33" s="7" t="n"/>
-      <c r="K33" s="9" t="n"/>
-      <c r="L33" s="7" t="n"/>
-      <c r="M33" s="9" t="n"/>
-      <c r="N33" s="7" t="n"/>
-      <c r="O33" s="9" t="n"/>
-      <c r="P33" s="7" t="n"/>
-      <c r="Q33" s="9" t="n"/>
-      <c r="R33" s="7" t="n"/>
-      <c r="S33" s="9" t="n"/>
-      <c r="T33" s="7" t="n"/>
-      <c r="U33" s="9" t="n"/>
-    </row>
-    <row r="34" ht="216" customHeight="1" s="142">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>근무 사유</t>
-        </is>
-      </c>
-      <c r="B34" s="159" t="n"/>
-      <c r="C34" s="81" t="n"/>
-      <c r="D34" s="159" t="n"/>
-      <c r="E34" s="81" t="n"/>
-      <c r="F34" s="159" t="n"/>
-      <c r="G34" s="81" t="n"/>
-      <c r="H34" s="159" t="n"/>
-      <c r="I34" s="81" t="n"/>
-      <c r="J34" s="159" t="n"/>
-      <c r="K34" s="81" t="n"/>
-      <c r="L34" s="159" t="n"/>
-      <c r="M34" s="81" t="n"/>
-      <c r="N34" s="159" t="n"/>
-      <c r="O34" s="81" t="n"/>
-      <c r="P34" s="159" t="n"/>
-      <c r="Q34" s="81" t="n"/>
-      <c r="R34" s="159" t="n"/>
-      <c r="S34" s="81" t="n"/>
-      <c r="T34" s="159" t="n"/>
-      <c r="U34" s="81" t="n"/>
-    </row>
-    <row r="35" ht="66" customHeight="1" s="142">
-      <c r="B35" s="154" t="n"/>
-      <c r="C35" s="80" t="n"/>
-      <c r="D35" s="80" t="n"/>
-      <c r="E35" s="80" t="n"/>
-      <c r="F35" s="80" t="n"/>
-      <c r="G35" s="80" t="n"/>
-      <c r="H35" s="80" t="n"/>
-      <c r="I35" s="80" t="n"/>
-      <c r="J35" s="80" t="n"/>
-      <c r="K35" s="80" t="n"/>
-      <c r="L35" s="80" t="n"/>
-      <c r="M35" s="80" t="n"/>
-      <c r="N35" s="80" t="n"/>
-      <c r="O35" s="80" t="n"/>
-      <c r="P35" s="80" t="n"/>
-      <c r="Q35" s="80" t="n"/>
-      <c r="R35" s="80" t="n"/>
-      <c r="S35" s="80" t="n"/>
-      <c r="T35" s="80" t="n"/>
-      <c r="U35" s="81" t="n"/>
-    </row>
-    <row r="36" ht="66" customHeight="1" s="142">
-      <c r="B36" s="138" t="n"/>
-      <c r="C36" s="139" t="n"/>
-      <c r="D36" s="139" t="n"/>
-      <c r="E36" s="139" t="n"/>
-      <c r="F36" s="139" t="n"/>
-      <c r="G36" s="139" t="n"/>
-      <c r="H36" s="139" t="n"/>
-      <c r="I36" s="139" t="n"/>
-      <c r="J36" s="139" t="n"/>
-      <c r="K36" s="139" t="n"/>
-      <c r="L36" s="139" t="n"/>
-      <c r="M36" s="139" t="n"/>
-      <c r="N36" s="139" t="n"/>
-      <c r="O36" s="139" t="n"/>
-      <c r="P36" s="139" t="n"/>
-      <c r="Q36" s="139" t="n"/>
-      <c r="R36" s="139" t="n"/>
-      <c r="S36" s="139" t="n"/>
-      <c r="T36" s="139" t="n"/>
-      <c r="U36" s="140" t="n"/>
-    </row>
-    <row r="37" ht="66" customHeight="1" s="142">
-      <c r="B37" s="106" t="n"/>
-      <c r="U37" s="143" t="n"/>
-    </row>
-    <row r="38" ht="66" customHeight="1" s="142">
-      <c r="B38" s="106" t="n"/>
-      <c r="U38" s="143" t="n"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="106" t="n"/>
-      <c r="U39" s="143" t="n"/>
-    </row>
-    <row r="40">
-      <c r="B40" s="106" t="n"/>
-      <c r="U40" s="143" t="n"/>
-    </row>
-    <row r="41">
-      <c r="B41" s="106" t="n"/>
-      <c r="U41" s="143" t="n"/>
-    </row>
-    <row r="42">
-      <c r="B42" s="106" t="n"/>
-      <c r="U42" s="143" t="n"/>
-    </row>
-    <row r="43">
-      <c r="B43" s="106" t="n"/>
-      <c r="U43" s="143" t="n"/>
-    </row>
-    <row r="44">
-      <c r="B44" s="106" t="n"/>
-      <c r="U44" s="143" t="n"/>
-    </row>
-    <row r="45">
-      <c r="B45" s="144" t="n"/>
-      <c r="C45" s="145" t="n"/>
-      <c r="D45" s="145" t="n"/>
-      <c r="E45" s="145" t="n"/>
-      <c r="F45" s="145" t="n"/>
-      <c r="G45" s="145" t="n"/>
-      <c r="H45" s="145" t="n"/>
-      <c r="I45" s="145" t="n"/>
-      <c r="J45" s="145" t="n"/>
-      <c r="K45" s="145" t="n"/>
-      <c r="L45" s="145" t="n"/>
-      <c r="M45" s="145" t="n"/>
-      <c r="N45" s="145" t="n"/>
-      <c r="O45" s="145" t="n"/>
-      <c r="P45" s="145" t="n"/>
-      <c r="Q45" s="145" t="n"/>
-      <c r="R45" s="145" t="n"/>
-      <c r="S45" s="145" t="n"/>
-      <c r="T45" s="145" t="n"/>
-      <c r="U45" s="146" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="78">
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="U2:U4"/>
-    <mergeCell ref="B1:U1"/>
-    <mergeCell ref="G2:G4"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="Q11:Q12"/>
-    <mergeCell ref="S2:S4"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="R18:S18"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="P26:Q26"/>
-    <mergeCell ref="B35:U35"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="P10:Q10"/>
-    <mergeCell ref="R10:S10"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="P34:Q34"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="R34:S34"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="T10:U10"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="I2:I4"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="K19:K20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="U19:U20"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="S11:S12"/>
-    <mergeCell ref="A27:A33"/>
-    <mergeCell ref="U11:U12"/>
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="O2:O4"/>
-    <mergeCell ref="Q2:Q4"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="Q19:Q20"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="A19:A25"/>
-    <mergeCell ref="O11:O12"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="T34:U34"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="K2:K4"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="S19:S20"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="R26:S26"/>
-    <mergeCell ref="T26:U26"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="M2:M4"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="A11:A17"/>
-    <mergeCell ref="P18:Q18"/>
-    <mergeCell ref="L34:M34"/>
-    <mergeCell ref="B36:U45"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="A2:A9"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="T18:U18"/>
-    <mergeCell ref="H26:I26"/>
-  </mergeCells>
-  <conditionalFormatting sqref="B3 B10 B11:U11 B17:B19 C19:U19 D3 D10 D17:D18 D26 F3 F10 F17:F19 F26 H3 H10 H17:H19 H26 J3 J10 J17:J19 J26 L3 L10 L17:L19 L26 N3 N10 N17:N19 N26 P3 R3 T3">
-    <cfRule type="expression" priority="54" dxfId="61">
-      <formula>ISNUMBER(MATCH(B3,#REF!, 0))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="53" dxfId="65">
-      <formula>OR(WEEKDAY(B3, 2)=6, WEEKDAY(B3, 2)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B4 B12 B20 D4 D12 D20 F4 F12 F20 H4 H12 H20 J4 J12 J20 L4 L12 L20 N4 N12 N20 P4 P12 P20 R4 R12 R20 T4 T12 T20">
-    <cfRule type="expression" priority="46" dxfId="65">
-      <formula>OR(WEEKDAY(B3, 2)=6, WEEKDAY(B3, 2)=7)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="45" dxfId="65">
-      <formula>ISNUMBER(MATCH(B3,#REF!, 0))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B26:B27">
-    <cfRule type="expression" priority="36" dxfId="61">
-      <formula>ISNUMBER(MATCH(B26,#REF!, 0))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="35" dxfId="65">
-      <formula>OR(WEEKDAY(B26, 2)=6, WEEKDAY(B26, 2)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B28 D28:E28">
-    <cfRule type="expression" priority="34" dxfId="65">
-      <formula>OR(WEEKDAY(B27, 2)=6, WEEKDAY(B27, 2)=7)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="33" dxfId="65">
-      <formula>ISNUMBER(MATCH(B27,#REF!, 0))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B34 D34 F34 H34 J34 L34 N34">
-    <cfRule type="expression" priority="9" dxfId="65">
-      <formula>OR(WEEKDAY(B34, 2)=6, WEEKDAY(B34, 2)=7)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="10" dxfId="61">
-      <formula>ISNUMBER(MATCH(B34,#REF!, 0))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C27:E27">
-    <cfRule type="expression" priority="1" dxfId="65">
-      <formula>OR(WEEKDAY(C27, 2)=6, WEEKDAY(C27, 2)=7)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="61">
-      <formula>ISNUMBER(MATCH(C27,#REF!, 0))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P10">
-    <cfRule type="expression" priority="27" dxfId="65">
-      <formula>OR(WEEKDAY(P10, 2)=6, WEEKDAY(P10, 2)=7)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="28" dxfId="61">
-      <formula>ISNUMBER(MATCH(P10,#REF!, 0))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P18">
-    <cfRule type="expression" priority="21" dxfId="65">
-      <formula>OR(WEEKDAY(P18, 2)=6, WEEKDAY(P18, 2)=7)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="22" dxfId="61">
-      <formula>ISNUMBER(MATCH(P18,#REF!, 0))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P26">
-    <cfRule type="expression" priority="15" dxfId="65">
-      <formula>OR(WEEKDAY(P26, 2)=6, WEEKDAY(P26, 2)=7)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="16" dxfId="61">
-      <formula>ISNUMBER(MATCH(P26,#REF!, 0))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P34">
-    <cfRule type="expression" priority="8" dxfId="61">
-      <formula>ISNUMBER(MATCH(P34,#REF!, 0))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="7" dxfId="65">
-      <formula>OR(WEEKDAY(P34, 2)=6, WEEKDAY(P34, 2)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R10">
-    <cfRule type="expression" priority="25" dxfId="65">
-      <formula>OR(WEEKDAY(R10, 2)=6, WEEKDAY(R10, 2)=7)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="26" dxfId="61">
-      <formula>ISNUMBER(MATCH(R10,#REF!, 0))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R18">
-    <cfRule type="expression" priority="20" dxfId="61">
-      <formula>ISNUMBER(MATCH(R18,#REF!, 0))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="19" dxfId="65">
-      <formula>OR(WEEKDAY(R18, 2)=6, WEEKDAY(R18, 2)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R26">
-    <cfRule type="expression" priority="13" dxfId="65">
-      <formula>OR(WEEKDAY(R26, 2)=6, WEEKDAY(R26, 2)=7)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="14" dxfId="61">
-      <formula>ISNUMBER(MATCH(R26,#REF!, 0))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R34">
-    <cfRule type="expression" priority="5" dxfId="65">
-      <formula>OR(WEEKDAY(R34, 2)=6, WEEKDAY(R34, 2)=7)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" dxfId="61">
-      <formula>ISNUMBER(MATCH(R34,#REF!, 0))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T10">
-    <cfRule type="expression" priority="24" dxfId="61">
-      <formula>ISNUMBER(MATCH(T10,#REF!, 0))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="23" dxfId="65">
-      <formula>OR(WEEKDAY(T10, 2)=6, WEEKDAY(T10, 2)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T18">
-    <cfRule type="expression" priority="18" dxfId="61">
-      <formula>ISNUMBER(MATCH(T18,#REF!, 0))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="17" dxfId="65">
-      <formula>OR(WEEKDAY(T18, 2)=6, WEEKDAY(T18, 2)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T26">
-    <cfRule type="expression" priority="11" dxfId="65">
-      <formula>OR(WEEKDAY(T26, 2)=6, WEEKDAY(T26, 2)=7)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="12" dxfId="61">
-      <formula>ISNUMBER(MATCH(T26,#REF!, 0))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T34">
-    <cfRule type="expression" priority="4" dxfId="61">
-      <formula>ISNUMBER(MATCH(T34,#REF!, 0))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="65">
-      <formula>OR(WEEKDAY(T34, 2)=6, WEEKDAY(T34, 2)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
     <tabColor rgb="FFFF0000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -8848,8 +7181,8 @@
     </row>
   </sheetData>
   <mergeCells count="76">
+    <mergeCell ref="AK26:AK28"/>
     <mergeCell ref="B47:C47"/>
-    <mergeCell ref="AK26:AK28"/>
     <mergeCell ref="AK41:AK43"/>
     <mergeCell ref="A8:A10"/>
     <mergeCell ref="A26:A28"/>

</xml_diff>